<commit_message>
Review of Steps 1-8: period severity bands, press releases, Titan notes
- thresholds.yaml: looser 'period' bands for prior / year-ago moves
  (79% of YoY moves graded High on one set of bands)
- press_release document type (table rebuilt in place, rows kept);
  Reliance press releases collected and searched by the cross-source check;
  Titan files none on NSE
- Titan: net debt no longer shown (gold metal loans); report notes for
  Titan and M&M in companies.yaml; sample model rebuilt (165 estimates)
- stale counts fixed in step records; docs/review_after_step8.md
- fresh rebuild reproduces the working database

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/sample_analyst_model.xlsx
+++ b/models/sample_analyst_model.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -959,27 +959,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Net debt</t>
+          <t>Jewellery secondary sales growth (overall)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>₹ crore</t>
+          <t>% YoY</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10053</v>
+        <v>47</v>
+      </c>
+      <c r="E20" t="n">
+        <v>37</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>net_debt</t>
+          <t>titan_secondary_growth</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jewellery secondary sales growth (overall)</t>
+          <t>Jewellery like-to-like secondary growth</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -988,35 +991,12 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>47</v>
+        <v>52.5</v>
       </c>
       <c r="E21" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F21" t="inlineStr">
-        <is>
-          <t>titan_secondary_growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Jewellery like-to-like secondary growth</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>% YoY</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="E22" t="n">
-        <v>34</v>
-      </c>
-      <c r="F22" t="inlineStr">
         <is>
           <t>titan_ltl_growth</t>
         </is>

</xml_diff>